<commit_message>
refactor processor registration and enhance index checker functionality
</commit_message>
<xml_diff>
--- a/test/res/task.xlsx
+++ b/test/res/task.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/codetypes/Desktop/Github/xlsx-exporter/test/res/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{68186292-A074-B04B-A2B6-FC43F57D1FF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CE6C439-CCEA-C948-96A3-D801C1C5A393}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="17700" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1101,7 +1101,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="723" uniqueCount="262">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="723" uniqueCount="263">
   <si>
     <t>id</t>
   </si>
@@ -1886,16 +1886,19 @@
     <t>$ &gt; 0 &amp;&amp; $ &lt; 20</t>
   </si>
   <si>
-    <t>#main.type=$&amp;key2=MAIN&amp;#main.condition=mainline_event</t>
-  </si>
-  <si>
-    <t>item#item.id=$.id</t>
-  </si>
-  <si>
-    <t>item#*.id=$.id</t>
-  </si>
-  <si>
-    <t>#define.value=$&amp;#define.key1=TASK_TYPE</t>
+    <t>#define.value&amp;key1=TASK_TYPE</t>
+  </si>
+  <si>
+    <t>$&amp;key2=MAIN==#main.type&amp;condition=mainline_event</t>
+  </si>
+  <si>
+    <t>$[*].id==item#item.id</t>
+  </si>
+  <si>
+    <t>$[*].id==item#*.id</t>
+  </si>
+  <si>
+    <t>$[*]==#branch.id</t>
   </si>
 </sst>
 </file>
@@ -3277,7 +3280,7 @@
         <v>13</v>
       </c>
       <c r="F5" s="33" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="G5" s="33" t="s">
         <v>13</v>
@@ -4159,7 +4162,7 @@
         <v>257</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>13</v>
@@ -4168,7 +4171,7 @@
         <v>101</v>
       </c>
       <c r="G4" s="2" t="s">
-        <v>102</v>
+        <v>262</v>
       </c>
       <c r="H4" s="2" t="s">
         <v>13</v>
@@ -6538,10 +6541,10 @@
         <v>13</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="J4" s="2" t="s">
         <v>13</v>

</xml_diff>

<commit_message>
feat: improve typedef workbook processing
</commit_message>
<xml_diff>
--- a/test/res/task.xlsx
+++ b/test/res/task.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Users\bite\Desktop\github\xlsx-exporter\test\res\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/codetypes/Desktop/Github/xlsx-exporter/test/res/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{718CF2AC-EFC2-455B-8CF6-1B8D933B94F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AAD05018-5370-084E-938D-63CC0632BB15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-32100" yWindow="1425" windowWidth="28395" windowHeight="18960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="30240" windowHeight="17680" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="define" sheetId="9" r:id="rId1"/>
@@ -1065,6 +1065,841 @@
     <author>Administrator</author>
   </authors>
   <commentList>
+    <comment ref="J5" authorId="0" shapeId="0" xr:uid="{2F804BCD-7389-9449-8311-A622B2319027}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>主线类型</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>type</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>：</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">        KILL_WOOD = 1,          -- </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>砍死一棵树</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">        KILL_FOOD = 2,          -- </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>割一片小麦</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">        RESCUS_SOLDIER = 3,     -- </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>解救士兵</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">        PICK_CHEST = 4,         -- </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>捡宝箱</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">        TALK_TO_NPC = 5,        -- </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>与</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>NPC</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>对话（可指定</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>Npc id:&lt;battle_npc&gt;</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>）</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">        KILL_MONSTER_TROOP = 6, -- </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>击杀怪物队伍（可指定队伍</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>id:&lt;monster.troop&gt;</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>）</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">        KILL_ANY_MONSTER_TROOP = 7, -- </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>击杀任意怪物队伍</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">        UPGRADE_BUILDING = 8,   -- </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>建造或者升级指定建筑（可指定建筑</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>id:&lt;battle_building&gt;</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>）</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">        UNLOCK_CLOUD = 9,       -- </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>解锁指定迷雾（可指定迷雾</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>id:&lt;1~n&gt;</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>）</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">        KILL_STONE = 10,         -- </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>采集一组矿</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">        COLLECT_ONE_WOOD = 11,  -- </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>采集一个木头资源</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">        COLLECT_ONE_FOOD = 12,  -- </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>采集一个粮食资源</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">        COLLECT_ONE_STONE = 13, -- </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>采集一个矿石资源</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">        COLLECT_ONE_ANY = 14,   -- </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>采集一个木头</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>/</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>粮食</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>/</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>矿石</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">        UNLOCK_ANY_CLOUD = 15,       -- </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>解锁任意指定迷雾</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">        FINISH_PLOT_THEATRE = 16  --</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>完成剧情对话，填</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>plot_theatre</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>表</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">ID 
+</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">        KILL_SCENARIO_MONSTER_TROOP = 18  -- </t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>击杀舞台剧怪物队伍</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>(</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t>可指定队伍</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color rgb="FF000000"/>
+            <rFont val="宋体"/>
+            <family val="3"/>
+            <charset val="134"/>
+          </rPr>
+          <t xml:space="preserve">id:&lt;monster.scenario_troop&gt;)
+</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments4.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Administrator</author>
+  </authors>
+  <commentList>
     <comment ref="I5" authorId="0" shapeId="0" xr:uid="{00000000-0006-0000-0700-000001000000}">
       <text>
         <r>
@@ -1101,7 +1936,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="270">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="745" uniqueCount="274">
   <si>
     <t>id</t>
   </si>
@@ -1925,17 +2760,29 @@
   <si>
     <t>@define;@stringify(task)</t>
     <phoneticPr fontId="8" type="noConversion"/>
+  </si>
+  <si>
+    <t>{kind:"kill_monster",count: 1,id:5}</t>
+  </si>
+  <si>
+    <t>{kind:"collect_coin",count:1,id:71001,duration:2}</t>
+  </si>
+  <si>
+    <t>task_args</t>
+  </si>
+  <si>
+    <t>TaskArgs?</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="11" x14ac:knownFonts="1">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
@@ -1964,7 +2811,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -1984,7 +2831,7 @@
     </font>
     <font>
       <sz val="9"/>
-      <name val="等线"/>
+      <name val="Calibri"/>
       <family val="3"/>
       <charset val="134"/>
       <scheme val="minor"/>
@@ -2264,7 +3111,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="3">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="常规 2" xfId="1" xr:uid="{00000000-0005-0000-0000-000031000000}"/>
     <cellStyle name="常规 3" xfId="2" xr:uid="{00000000-0005-0000-0000-000032000000}"/>
   </cellStyles>
@@ -3190,17 +4037,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I24"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="2" max="2" width="14.625" customWidth="1"/>
-    <col min="3" max="3" width="16.625" customWidth="1"/>
-    <col min="4" max="4" width="25.625" customWidth="1"/>
-    <col min="5" max="5" width="45.875" customWidth="1"/>
-    <col min="6" max="6" width="18.625" customWidth="1"/>
-    <col min="8" max="9" width="12.625" customWidth="1"/>
+    <col min="2" max="2" width="14.6640625" customWidth="1"/>
+    <col min="3" max="3" width="16.6640625" customWidth="1"/>
+    <col min="4" max="4" width="25.6640625" customWidth="1"/>
+    <col min="5" max="5" width="45.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.6640625" customWidth="1"/>
+    <col min="8" max="9" width="12.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:9">
       <c r="A1" s="40" t="s">
         <v>269</v>
       </c>
@@ -3210,7 +4057,7 @@
       <c r="E1" s="41"/>
       <c r="F1" s="41"/>
     </row>
-    <row r="2" spans="1:9" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:9" ht="16">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -3239,7 +4086,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="3" spans="1:9" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:9" ht="16">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -3268,7 +4115,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="4" spans="1:9" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:9" ht="16">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
@@ -3283,7 +4130,7 @@
       <c r="H4" s="32"/>
       <c r="I4" s="32"/>
     </row>
-    <row r="5" spans="1:9" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:9" ht="16">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
@@ -3312,7 +4159,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:9" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:9" ht="16">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -3329,7 +4176,7 @@
       <c r="H6" s="32"/>
       <c r="I6" s="32"/>
     </row>
-    <row r="7" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" ht="16">
       <c r="A7" s="21" t="s">
         <v>17</v>
       </c>
@@ -3358,7 +4205,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="8" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9" ht="16">
       <c r="A8" s="21" t="s">
         <v>17</v>
       </c>
@@ -3381,7 +4228,7 @@
       <c r="H8" s="33"/>
       <c r="I8" s="33"/>
     </row>
-    <row r="9" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9" ht="16">
       <c r="A9" s="21" t="s">
         <v>17</v>
       </c>
@@ -3404,7 +4251,7 @@
       <c r="H9" s="33"/>
       <c r="I9" s="33"/>
     </row>
-    <row r="10" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9" ht="16">
       <c r="A10" s="21" t="s">
         <v>17</v>
       </c>
@@ -3427,7 +4274,7 @@
       <c r="H10" s="33"/>
       <c r="I10" s="33"/>
     </row>
-    <row r="11" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9" ht="16">
       <c r="A11" s="21" t="s">
         <v>17</v>
       </c>
@@ -3450,7 +4297,7 @@
       <c r="H11" s="33"/>
       <c r="I11" s="33"/>
     </row>
-    <row r="12" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9" ht="16">
       <c r="A12" s="21" t="s">
         <v>17</v>
       </c>
@@ -3473,7 +4320,7 @@
       <c r="H12" s="33"/>
       <c r="I12" s="33"/>
     </row>
-    <row r="13" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9" ht="16">
       <c r="A13" s="21" t="s">
         <v>17</v>
       </c>
@@ -3496,7 +4343,7 @@
       <c r="H13" s="33"/>
       <c r="I13" s="33"/>
     </row>
-    <row r="14" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9" ht="16">
       <c r="A14" s="21" t="s">
         <v>17</v>
       </c>
@@ -3523,7 +4370,7 @@
       </c>
       <c r="I14" s="33"/>
     </row>
-    <row r="15" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9" ht="16">
       <c r="A15" s="21" t="s">
         <v>17</v>
       </c>
@@ -3546,7 +4393,7 @@
       <c r="H15" s="33"/>
       <c r="I15" s="33"/>
     </row>
-    <row r="16" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9" ht="16">
       <c r="A16" s="21" t="s">
         <v>17</v>
       </c>
@@ -3569,7 +4416,7 @@
       <c r="H16" s="33"/>
       <c r="I16" s="33"/>
     </row>
-    <row r="17" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9" ht="16">
       <c r="A17" s="21" t="s">
         <v>17</v>
       </c>
@@ -3592,7 +4439,7 @@
       <c r="H17" s="33"/>
       <c r="I17" s="33"/>
     </row>
-    <row r="18" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9" ht="16">
       <c r="A18" s="21" t="s">
         <v>17</v>
       </c>
@@ -3615,7 +4462,7 @@
       <c r="H18" s="33"/>
       <c r="I18" s="33"/>
     </row>
-    <row r="19" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9" ht="16">
       <c r="A19" s="21" t="s">
         <v>17</v>
       </c>
@@ -3638,7 +4485,7 @@
       <c r="H19" s="33"/>
       <c r="I19" s="33"/>
     </row>
-    <row r="20" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9" ht="16">
       <c r="A20" s="21" t="s">
         <v>17</v>
       </c>
@@ -3665,7 +4512,7 @@
       </c>
       <c r="I20" s="33"/>
     </row>
-    <row r="21" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:9" ht="16">
       <c r="A21" s="21" t="s">
         <v>17</v>
       </c>
@@ -3688,7 +4535,7 @@
       <c r="H21" s="33"/>
       <c r="I21" s="33"/>
     </row>
-    <row r="22" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:9" ht="16">
       <c r="A22" s="21" t="s">
         <v>17</v>
       </c>
@@ -3711,7 +4558,7 @@
       <c r="H22" s="33"/>
       <c r="I22" s="33"/>
     </row>
-    <row r="23" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:9" ht="16">
       <c r="A23" s="21" t="s">
         <v>17</v>
       </c>
@@ -3734,7 +4581,7 @@
       <c r="H23" s="33"/>
       <c r="I23" s="33"/>
     </row>
-    <row r="24" spans="1:9" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:9" ht="16">
       <c r="A24" s="21" t="s">
         <v>17</v>
       </c>
@@ -3770,16 +4617,16 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{984B885C-48D0-4D9B-AAB3-39C5F463E278}">
   <dimension ref="A1:E10"/>
-  <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9" style="39"/>
     <col min="2" max="2" width="32.5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="6.5" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.6640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="49" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5">
       <c r="A1" s="42" t="s">
         <v>251</v>
       </c>
@@ -3788,7 +4635,7 @@
       <c r="D1" s="43"/>
       <c r="E1" s="43"/>
     </row>
-    <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:5" ht="16">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -3805,7 +4652,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" ht="16">
       <c r="A3" s="1" t="s">
         <v>9</v>
       </c>
@@ -3822,7 +4669,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" ht="16">
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
@@ -3831,7 +4678,7 @@
       <c r="D4" s="2"/>
       <c r="E4" s="2"/>
     </row>
-    <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" ht="16">
       <c r="A5" s="1" t="s">
         <v>14</v>
       </c>
@@ -3848,7 +4695,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" ht="16">
       <c r="A6" s="1" t="s">
         <v>15</v>
       </c>
@@ -3865,7 +4712,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:5">
       <c r="A7" s="39" t="s">
         <v>17</v>
       </c>
@@ -3882,7 +4729,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:5">
       <c r="A8" s="39" t="s">
         <v>17</v>
       </c>
@@ -3899,7 +4746,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:5">
       <c r="A9" s="39" t="s">
         <v>17</v>
       </c>
@@ -3917,7 +4764,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:5">
       <c r="A10" s="39" t="s">
         <v>17</v>
       </c>
@@ -3948,26 +4795,26 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:X17"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="17.125" style="9" customWidth="1"/>
-    <col min="2" max="2" width="17.875" style="9" customWidth="1"/>
-    <col min="3" max="4" width="15.125" style="9" customWidth="1"/>
-    <col min="5" max="5" width="26.875" style="9" customWidth="1"/>
-    <col min="6" max="6" width="19.75" style="9" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.125" style="9" customWidth="1"/>
-    <col min="8" max="8" width="23.125" style="9" customWidth="1"/>
+    <col min="1" max="1" width="17.1640625" style="9" customWidth="1"/>
+    <col min="2" max="2" width="17.83203125" style="9" customWidth="1"/>
+    <col min="3" max="4" width="15.1640625" style="9" customWidth="1"/>
+    <col min="5" max="5" width="26.83203125" style="9" customWidth="1"/>
+    <col min="6" max="6" width="19.6640625" style="9" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.1640625" style="9" customWidth="1"/>
+    <col min="8" max="8" width="23.1640625" style="9" customWidth="1"/>
     <col min="9" max="9" width="5" style="9" customWidth="1"/>
-    <col min="10" max="10" width="46.125" style="9" customWidth="1"/>
+    <col min="10" max="10" width="46.1640625" style="9" customWidth="1"/>
     <col min="11" max="11" width="31.5" style="9" customWidth="1"/>
     <col min="12" max="12" width="8" style="9" customWidth="1"/>
-    <col min="13" max="13" width="73.625" style="9" customWidth="1"/>
-    <col min="14" max="14" width="13.125" style="9" customWidth="1"/>
-    <col min="15" max="15" width="20.625" style="8" customWidth="1"/>
+    <col min="13" max="13" width="73.6640625" style="9" customWidth="1"/>
+    <col min="14" max="14" width="13.1640625" style="9" customWidth="1"/>
+    <col min="15" max="15" width="20.6640625" style="8" customWidth="1"/>
     <col min="16" max="16384" width="9" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:24">
       <c r="A1" s="21" t="s">
         <v>0</v>
       </c>
@@ -4041,7 +4888,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:24">
       <c r="A2" s="21" t="s">
         <v>22</v>
       </c>
@@ -4115,7 +4962,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:24">
       <c r="A3" s="21" t="s">
         <v>12</v>
       </c>
@@ -4171,7 +5018,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:24">
       <c r="A4" s="21" t="s">
         <v>14</v>
       </c>
@@ -4245,7 +5092,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:24">
       <c r="A5" s="21" t="s">
         <v>15</v>
       </c>
@@ -4317,7 +5164,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:24" ht="17">
       <c r="A6" s="22">
         <v>1001</v>
       </c>
@@ -4384,7 +5231,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:24">
       <c r="A7" s="22">
         <v>1002</v>
       </c>
@@ -4444,7 +5291,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:24" ht="17">
       <c r="A8" s="22">
         <v>1003</v>
       </c>
@@ -4509,7 +5356,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:24" ht="17">
       <c r="A9" s="22">
         <v>1014</v>
       </c>
@@ -4571,7 +5418,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:24">
       <c r="A10" s="22">
         <v>100301</v>
       </c>
@@ -4641,7 +5488,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:24" ht="17">
       <c r="A11" s="22">
         <v>100302</v>
       </c>
@@ -4701,7 +5548,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:24" s="20" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:24" s="20" customFormat="1" ht="17">
       <c r="A12" s="24">
         <v>100303</v>
       </c>
@@ -4761,7 +5608,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:24" ht="17">
       <c r="A13" s="22">
         <v>100001</v>
       </c>
@@ -4821,7 +5668,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:24">
       <c r="A14" s="22">
         <v>100002</v>
       </c>
@@ -4881,7 +5728,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:24">
       <c r="A15" s="22">
         <v>100003</v>
       </c>
@@ -4943,7 +5790,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:24" ht="17">
       <c r="A16" s="22">
         <v>100304</v>
       </c>
@@ -5003,7 +5850,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:23" ht="17">
       <c r="A17" s="22">
         <v>1013</v>
       </c>
@@ -5075,27 +5922,27 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:X16"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="17.125" style="9" customWidth="1"/>
-    <col min="2" max="3" width="17.875" style="9" customWidth="1"/>
-    <col min="4" max="5" width="15.125" style="9" customWidth="1"/>
-    <col min="6" max="6" width="19.875" style="9" customWidth="1"/>
+    <col min="1" max="1" width="17.1640625" style="9" customWidth="1"/>
+    <col min="2" max="3" width="17.83203125" style="9" customWidth="1"/>
+    <col min="4" max="5" width="15.1640625" style="9" customWidth="1"/>
+    <col min="6" max="6" width="19.83203125" style="9" customWidth="1"/>
     <col min="7" max="7" width="28" style="9" customWidth="1"/>
-    <col min="8" max="8" width="15.125" style="9" customWidth="1"/>
-    <col min="9" max="9" width="23.125" style="9" customWidth="1"/>
-    <col min="10" max="10" width="16.125" style="9" customWidth="1"/>
-    <col min="11" max="11" width="63.125" style="9" customWidth="1"/>
-    <col min="12" max="12" width="8.875" style="9" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="20.125" style="9" customWidth="1"/>
-    <col min="14" max="14" width="13.125" style="9" customWidth="1"/>
+    <col min="8" max="8" width="15.1640625" style="9" customWidth="1"/>
+    <col min="9" max="9" width="23.1640625" style="9" customWidth="1"/>
+    <col min="10" max="10" width="16.1640625" style="9" customWidth="1"/>
+    <col min="11" max="11" width="63.1640625" style="9" customWidth="1"/>
+    <col min="12" max="12" width="8.83203125" style="9" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.1640625" style="9" customWidth="1"/>
+    <col min="14" max="14" width="13.1640625" style="9" customWidth="1"/>
     <col min="15" max="15" width="9" style="9"/>
-    <col min="16" max="16" width="13.125" style="9" customWidth="1"/>
+    <col min="16" max="16" width="13.1640625" style="9" customWidth="1"/>
     <col min="17" max="17" width="11" style="9" customWidth="1"/>
     <col min="18" max="16384" width="9" style="9"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:24">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -5166,7 +6013,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="2" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:24">
       <c r="A2" s="1" t="s">
         <v>22</v>
       </c>
@@ -5237,7 +6084,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:24">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -5289,7 +6136,7 @@
       </c>
       <c r="X3" s="1"/>
     </row>
-    <row r="4" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:24">
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
@@ -5361,7 +6208,7 @@
       </c>
       <c r="X4" s="12"/>
     </row>
-    <row r="5" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:24">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
@@ -5430,7 +6277,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="6" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:24">
       <c r="A6" s="9">
         <f t="shared" ref="A6:A16" si="0">200000+C6*100+D6</f>
         <v>200101</v>
@@ -5490,7 +6337,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="7" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:24">
       <c r="A7" s="9">
         <f t="shared" si="0"/>
         <v>200102</v>
@@ -5549,7 +6396,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:24">
       <c r="A8" s="9">
         <f t="shared" si="0"/>
         <v>200103</v>
@@ -5611,7 +6458,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="9" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:24">
       <c r="A9" s="9">
         <f t="shared" si="0"/>
         <v>200104</v>
@@ -5670,7 +6517,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:24">
       <c r="A10" s="9">
         <f t="shared" si="0"/>
         <v>200105</v>
@@ -5729,7 +6576,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="11" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:24">
       <c r="A11" s="9">
         <f t="shared" si="0"/>
         <v>200106</v>
@@ -5788,7 +6635,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:24">
       <c r="A12" s="9">
         <f t="shared" si="0"/>
         <v>200107</v>
@@ -5847,7 +6694,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="13" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:24">
       <c r="A13" s="9">
         <f t="shared" si="0"/>
         <v>200201</v>
@@ -5909,7 +6756,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:24">
       <c r="A14" s="9">
         <f t="shared" si="0"/>
         <v>200202</v>
@@ -5971,7 +6818,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="15" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:24">
       <c r="A15" s="9">
         <f t="shared" si="0"/>
         <v>200203</v>
@@ -6033,7 +6880,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:24" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:24">
       <c r="A16" s="9">
         <f t="shared" si="0"/>
         <v>200204</v>
@@ -6101,21 +6948,22 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <tabColor theme="5" tint="0.39915158543656726"/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:J19"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="2" width="17.125" customWidth="1"/>
-    <col min="3" max="3" width="15.125" style="9" customWidth="1"/>
-    <col min="4" max="7" width="17.125" customWidth="1"/>
-    <col min="8" max="8" width="20.125" customWidth="1"/>
-    <col min="9" max="9" width="13.125" style="9" customWidth="1"/>
+    <col min="1" max="2" width="17.1640625" customWidth="1"/>
+    <col min="3" max="3" width="15.1640625" style="9" customWidth="1"/>
+    <col min="4" max="7" width="17.1640625" customWidth="1"/>
+    <col min="8" max="8" width="20.1640625" customWidth="1"/>
+    <col min="9" max="9" width="13.1640625" style="9" customWidth="1"/>
+    <col min="10" max="10" width="39.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6143,8 +6991,11 @@
       <c r="I1" s="2" t="s">
         <v>81</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J1" s="2" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
       <c r="A2" s="1" t="s">
         <v>22</v>
       </c>
@@ -6172,8 +7023,11 @@
       <c r="I2" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J2" s="2" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -6193,8 +7047,9 @@
       <c r="I3" s="2" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J3" s="2"/>
+    </row>
+    <row r="4" spans="1:10">
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
@@ -6222,8 +7077,11 @@
       <c r="I4" s="2" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J4" s="2" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
@@ -6251,8 +7109,11 @@
       <c r="I5" s="7" t="s">
         <v>111</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J5" s="13" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
       <c r="A6" s="4" t="s">
         <v>175</v>
       </c>
@@ -6280,8 +7141,11 @@
       <c r="I6" s="6">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J6" s="19" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
       <c r="A7" s="4" t="s">
         <v>181</v>
       </c>
@@ -6309,8 +7173,11 @@
       <c r="I7" s="6">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="J7" s="8" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
       <c r="A8" s="4" t="s">
         <v>186</v>
       </c>
@@ -6339,7 +7206,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10">
       <c r="A9" s="4" t="s">
         <v>191</v>
       </c>
@@ -6368,7 +7235,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10">
       <c r="A10" s="4"/>
       <c r="B10" s="5"/>
       <c r="C10" s="6"/>
@@ -6379,7 +7246,7 @@
       <c r="H10" s="6"/>
       <c r="I10" s="6"/>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10">
       <c r="A11" s="4"/>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
@@ -6390,7 +7257,7 @@
       <c r="H11" s="6"/>
       <c r="I11" s="6"/>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10">
       <c r="A12" s="4"/>
       <c r="B12" s="5"/>
       <c r="C12" s="6"/>
@@ -6401,7 +7268,7 @@
       <c r="H12" s="6"/>
       <c r="I12" s="6"/>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10">
       <c r="A13" s="4"/>
       <c r="B13" s="5"/>
       <c r="C13" s="6"/>
@@ -6412,7 +7279,7 @@
       <c r="H13" s="6"/>
       <c r="I13" s="6"/>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10">
       <c r="A14" s="4"/>
       <c r="B14" s="5"/>
       <c r="C14" s="6"/>
@@ -6423,7 +7290,7 @@
       <c r="H14" s="6"/>
       <c r="I14" s="6"/>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10">
       <c r="A15" s="4"/>
       <c r="B15" s="5"/>
       <c r="C15" s="6"/>
@@ -6434,7 +7301,7 @@
       <c r="H15" s="6"/>
       <c r="I15" s="6"/>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10">
       <c r="A16" s="4"/>
       <c r="B16" s="5"/>
       <c r="C16" s="6"/>
@@ -6445,7 +7312,7 @@
       <c r="H16" s="6"/>
       <c r="I16" s="6"/>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9">
       <c r="A17" s="4"/>
       <c r="B17" s="5"/>
       <c r="C17" s="6"/>
@@ -6456,7 +7323,7 @@
       <c r="H17" s="6"/>
       <c r="I17" s="6"/>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9">
       <c r="A18" s="4"/>
       <c r="B18" s="5"/>
       <c r="C18" s="6"/>
@@ -6467,7 +7334,7 @@
       <c r="H18" s="6"/>
       <c r="I18" s="6"/>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9">
       <c r="A19" s="4"/>
       <c r="B19" s="5"/>
       <c r="C19" s="6"/>
@@ -6482,6 +7349,7 @@
   <phoneticPr fontId="8" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -6491,17 +7359,17 @@
     <tabColor theme="5" tint="0.39915158543656726"/>
   </sheetPr>
   <dimension ref="A1:J19"/>
-  <sheetFormatPr defaultColWidth="17.125" defaultRowHeight="16.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="17.1640625" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="2" width="17.125" customWidth="1"/>
-    <col min="3" max="3" width="15.125" style="9" customWidth="1"/>
-    <col min="4" max="7" width="17.125" customWidth="1"/>
-    <col min="8" max="9" width="25.625" customWidth="1"/>
-    <col min="10" max="10" width="13.125" style="9" customWidth="1"/>
-    <col min="11" max="16377" width="17.125" customWidth="1"/>
+    <col min="1" max="2" width="17.1640625" customWidth="1"/>
+    <col min="3" max="3" width="15.1640625" style="9" customWidth="1"/>
+    <col min="4" max="7" width="17.1640625" customWidth="1"/>
+    <col min="8" max="9" width="25.6640625" customWidth="1"/>
+    <col min="10" max="10" width="13.1640625" style="9" customWidth="1"/>
+    <col min="11" max="16377" width="17.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="16.5">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6533,7 +7401,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="16.5">
       <c r="A2" s="1" t="s">
         <v>22</v>
       </c>
@@ -6565,7 +7433,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" ht="16.5">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -6587,7 +7455,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" ht="16.5">
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
@@ -6619,7 +7487,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" ht="16.5">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
@@ -6651,7 +7519,7 @@
         <v>111</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10">
       <c r="A6" s="4" t="s">
         <v>198</v>
       </c>
@@ -6683,7 +7551,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10">
       <c r="A7" s="4" t="s">
         <v>200</v>
       </c>
@@ -6715,7 +7583,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10">
       <c r="A8" s="4" t="s">
         <v>204</v>
       </c>
@@ -6747,7 +7615,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10">
       <c r="A9" s="4" t="s">
         <v>208</v>
       </c>
@@ -6779,7 +7647,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10">
       <c r="A10" s="4"/>
       <c r="B10" s="5"/>
       <c r="C10" s="6"/>
@@ -6791,7 +7659,7 @@
       <c r="I10" s="6"/>
       <c r="J10" s="6"/>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10">
       <c r="A11" s="4"/>
       <c r="B11" s="5"/>
       <c r="C11" s="6"/>
@@ -6803,7 +7671,7 @@
       <c r="I11" s="6"/>
       <c r="J11" s="6"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10">
       <c r="A12" s="4"/>
       <c r="B12" s="5"/>
       <c r="C12" s="6"/>
@@ -6815,7 +7683,7 @@
       <c r="I12" s="6"/>
       <c r="J12" s="6"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10">
       <c r="A13" s="4"/>
       <c r="B13" s="5"/>
       <c r="C13" s="6"/>
@@ -6827,7 +7695,7 @@
       <c r="I13" s="6"/>
       <c r="J13" s="6"/>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10">
       <c r="A14" s="4"/>
       <c r="B14" s="5"/>
       <c r="C14" s="6"/>
@@ -6839,19 +7707,19 @@
       <c r="I14" s="6"/>
       <c r="J14" s="6"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10">
       <c r="J15" s="6"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10">
       <c r="J16" s="6"/>
     </row>
-    <row r="17" spans="10:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="10:10">
       <c r="J17" s="6"/>
     </row>
-    <row r="18" spans="10:10" x14ac:dyDescent="0.35">
+    <row r="18" spans="10:10">
       <c r="J18" s="6"/>
     </row>
-    <row r="19" spans="10:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="10:10">
       <c r="J19" s="6"/>
     </row>
   </sheetData>
@@ -6864,18 +7732,18 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:L9"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="4" max="4" width="10.625" customWidth="1"/>
+    <col min="4" max="4" width="10.6640625" customWidth="1"/>
     <col min="5" max="5" width="29" customWidth="1"/>
-    <col min="6" max="6" width="20.875" customWidth="1"/>
-    <col min="7" max="7" width="16.625" customWidth="1"/>
-    <col min="9" max="9" width="35.625" customWidth="1"/>
-    <col min="10" max="10" width="21.875" customWidth="1"/>
+    <col min="6" max="6" width="20.83203125" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" customWidth="1"/>
+    <col min="9" max="9" width="35.6640625" customWidth="1"/>
+    <col min="10" max="10" width="21.83203125" customWidth="1"/>
     <col min="12" max="12" width="52" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:12" ht="16">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -6913,7 +7781,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="2" spans="1:12" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:12" ht="16">
       <c r="A2" s="1" t="s">
         <v>22</v>
       </c>
@@ -6951,7 +7819,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="3" spans="1:12" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:12" ht="16">
       <c r="A3" s="1" t="s">
         <v>12</v>
       </c>
@@ -6975,7 +7843,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:12" ht="16">
       <c r="A4" s="1" t="s">
         <v>14</v>
       </c>
@@ -7013,7 +7881,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="16.5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:12" ht="16">
       <c r="A5" s="1" t="s">
         <v>15</v>
       </c>
@@ -7051,7 +7919,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="6" spans="1:12" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" ht="16">
       <c r="A6" s="4" t="s">
         <v>213</v>
       </c>
@@ -7085,7 +7953,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="7" spans="1:12" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" ht="16">
       <c r="A7" s="4" t="s">
         <v>219</v>
       </c>
@@ -7119,7 +7987,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="8" spans="1:12" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" ht="16">
       <c r="A8" s="4" t="s">
         <v>224</v>
       </c>
@@ -7153,7 +8021,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="9" spans="1:12" ht="16.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" ht="16">
       <c r="A9" s="4" t="s">
         <v>229</v>
       </c>

</xml_diff>